<commit_message>
fix(carton): make opening imports reversible and correct collaboration state
</commit_message>
<xml_diff>
--- a/backend/app/templates/spreadsheet_merge/carton-history-inventory-import-template.xlsx
+++ b/backend/app/templates/spreadsheet_merge/carton-history-inventory-import-template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="期初库存导入" sheetId="1" r:id="R5d83af78c56a4e2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写示例" sheetId="2" r:id="Rd28f17bf197846ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="Rc1e6b3bad66c462c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="期初库存导入" sheetId="1" r:id="R114ec75d65634e23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写示例" sheetId="2" r:id="R24e31c645cfe4a1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="R7768ca7fad1b4a5c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -159,7 +159,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="69">
+  <x:cellXfs count="72">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -348,6 +348,13 @@
     <x:xf numFmtId="203" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -611,6 +618,7 @@
     <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="16" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="26" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
@@ -635,10 +643,13 @@
       <x:c r="K1" s="42"/>
       <x:c r="L1" s="42"/>
       <x:c r="M1" s="42"/>
+      <x:c r="P1" s="42" t="str">
+        <x:v>客户选填</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="42" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>PO</x:v>
+        <x:v>合同号</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
         <x:v>货号</x:v>
@@ -681,6 +692,9 @@
       </x:c>
       <x:c r="O2" s="68" t="str">
         <x:v>入库时间</x:v>
+      </x:c>
+      <x:c r="P2" s="9" t="str">
+        <x:v>客户</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
@@ -699,6 +713,7 @@
       <x:c r="M3" s="39"/>
       <x:c r="N3" s="65" t="str"/>
       <x:c r="O3" s="67" t="str"/>
+      <x:c r="P3" s="36"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="19"/>
@@ -716,6 +731,7 @@
       <x:c r="M4" s="40"/>
       <x:c r="N4" s="65" t="str"/>
       <x:c r="O4" s="67" t="str"/>
+      <x:c r="P4" s="37"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="19"/>
@@ -733,6 +749,7 @@
       <x:c r="M5" s="40"/>
       <x:c r="N5" s="65" t="str"/>
       <x:c r="O5" s="67" t="str"/>
+      <x:c r="P5" s="37"/>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="19"/>
@@ -750,6 +767,7 @@
       <x:c r="M6" s="40"/>
       <x:c r="N6" s="65" t="str"/>
       <x:c r="O6" s="67" t="str"/>
+      <x:c r="P6" s="37"/>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
       <x:c r="A7" s="19"/>
@@ -767,6 +785,7 @@
       <x:c r="M7" s="40"/>
       <x:c r="N7" s="65" t="str"/>
       <x:c r="O7" s="67" t="str"/>
+      <x:c r="P7" s="37"/>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
       <x:c r="A8" s="19"/>
@@ -784,6 +803,7 @@
       <x:c r="M8" s="40"/>
       <x:c r="N8" s="65" t="str"/>
       <x:c r="O8" s="67" t="str"/>
+      <x:c r="P8" s="37"/>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
       <x:c r="A9" s="19"/>
@@ -801,6 +821,7 @@
       <x:c r="M9" s="40"/>
       <x:c r="N9" s="65" t="str"/>
       <x:c r="O9" s="67" t="str"/>
+      <x:c r="P9" s="37"/>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
       <x:c r="A10" s="19"/>
@@ -818,6 +839,7 @@
       <x:c r="M10" s="40"/>
       <x:c r="N10" s="65" t="str"/>
       <x:c r="O10" s="67" t="str"/>
+      <x:c r="P10" s="37"/>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
       <x:c r="A11" s="19"/>
@@ -835,6 +857,7 @@
       <x:c r="M11" s="40"/>
       <x:c r="N11" s="65" t="str"/>
       <x:c r="O11" s="67" t="str"/>
+      <x:c r="P11" s="37"/>
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
       <x:c r="A12" s="19"/>
@@ -852,6 +875,7 @@
       <x:c r="M12" s="40"/>
       <x:c r="N12" s="65" t="str"/>
       <x:c r="O12" s="67" t="str"/>
+      <x:c r="P12" s="37"/>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="19"/>
@@ -869,6 +893,7 @@
       <x:c r="M13" s="40"/>
       <x:c r="N13" s="65" t="str"/>
       <x:c r="O13" s="67" t="str"/>
+      <x:c r="P13" s="37"/>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
       <x:c r="A14" s="19"/>
@@ -886,6 +911,7 @@
       <x:c r="M14" s="40"/>
       <x:c r="N14" s="65" t="str"/>
       <x:c r="O14" s="67" t="str"/>
+      <x:c r="P14" s="37"/>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
       <x:c r="A15" s="19"/>
@@ -903,6 +929,7 @@
       <x:c r="M15" s="40"/>
       <x:c r="N15" s="65" t="str"/>
       <x:c r="O15" s="67" t="str"/>
+      <x:c r="P15" s="37"/>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
       <x:c r="A16" s="19"/>
@@ -920,6 +947,7 @@
       <x:c r="M16" s="40"/>
       <x:c r="N16" s="65" t="str"/>
       <x:c r="O16" s="67" t="str"/>
+      <x:c r="P16" s="37"/>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="19"/>
@@ -937,6 +965,7 @@
       <x:c r="M17" s="40"/>
       <x:c r="N17" s="65" t="str"/>
       <x:c r="O17" s="67" t="str"/>
+      <x:c r="P17" s="37"/>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
       <x:c r="A18" s="19"/>
@@ -954,6 +983,7 @@
       <x:c r="M18" s="40"/>
       <x:c r="N18" s="65" t="str"/>
       <x:c r="O18" s="67" t="str"/>
+      <x:c r="P18" s="37"/>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
       <x:c r="A19" s="19"/>
@@ -971,6 +1001,7 @@
       <x:c r="M19" s="40"/>
       <x:c r="N19" s="65" t="str"/>
       <x:c r="O19" s="67" t="str"/>
+      <x:c r="P19" s="37"/>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
       <x:c r="A20" s="19"/>
@@ -988,6 +1019,7 @@
       <x:c r="M20" s="40"/>
       <x:c r="N20" s="65" t="str"/>
       <x:c r="O20" s="67" t="str"/>
+      <x:c r="P20" s="37"/>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
       <x:c r="A21" s="19"/>
@@ -1005,6 +1037,7 @@
       <x:c r="M21" s="40"/>
       <x:c r="N21" s="65" t="str"/>
       <x:c r="O21" s="67" t="str"/>
+      <x:c r="P21" s="37"/>
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="19"/>
@@ -1022,6 +1055,7 @@
       <x:c r="M22" s="40"/>
       <x:c r="N22" s="65" t="str"/>
       <x:c r="O22" s="67" t="str"/>
+      <x:c r="P22" s="37"/>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
       <x:c r="A23" s="19"/>
@@ -1039,6 +1073,7 @@
       <x:c r="M23" s="40"/>
       <x:c r="N23" s="65" t="str"/>
       <x:c r="O23" s="67" t="str"/>
+      <x:c r="P23" s="37"/>
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
       <x:c r="A24" s="19"/>
@@ -1056,6 +1091,7 @@
       <x:c r="M24" s="40"/>
       <x:c r="N24" s="65" t="str"/>
       <x:c r="O24" s="67" t="str"/>
+      <x:c r="P24" s="37"/>
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
       <x:c r="A25" s="19"/>
@@ -1073,6 +1109,7 @@
       <x:c r="M25" s="40"/>
       <x:c r="N25" s="65" t="str"/>
       <x:c r="O25" s="67" t="str"/>
+      <x:c r="P25" s="37"/>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
       <x:c r="A26" s="19"/>
@@ -1090,6 +1127,7 @@
       <x:c r="M26" s="40"/>
       <x:c r="N26" s="65" t="str"/>
       <x:c r="O26" s="67" t="str"/>
+      <x:c r="P26" s="37"/>
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
       <x:c r="A27" s="19"/>
@@ -1107,6 +1145,7 @@
       <x:c r="M27" s="40"/>
       <x:c r="N27" s="65" t="str"/>
       <x:c r="O27" s="67" t="str"/>
+      <x:c r="P27" s="37"/>
     </x:row>
     <x:row r="28" ht="30" customHeight="1">
       <x:c r="A28" s="19"/>
@@ -1124,6 +1163,7 @@
       <x:c r="M28" s="40"/>
       <x:c r="N28" s="65" t="str"/>
       <x:c r="O28" s="67" t="str"/>
+      <x:c r="P28" s="37"/>
     </x:row>
     <x:row r="29" ht="30" customHeight="1">
       <x:c r="A29" s="19"/>
@@ -1141,6 +1181,7 @@
       <x:c r="M29" s="40"/>
       <x:c r="N29" s="65" t="str"/>
       <x:c r="O29" s="67" t="str"/>
+      <x:c r="P29" s="37"/>
     </x:row>
     <x:row r="30" ht="30" customHeight="1">
       <x:c r="A30" s="19"/>
@@ -1158,6 +1199,7 @@
       <x:c r="M30" s="40"/>
       <x:c r="N30" s="65" t="str"/>
       <x:c r="O30" s="67" t="str"/>
+      <x:c r="P30" s="37"/>
     </x:row>
     <x:row r="31" ht="30" customHeight="1">
       <x:c r="A31" s="19"/>
@@ -1175,6 +1217,7 @@
       <x:c r="M31" s="40"/>
       <x:c r="N31" s="65" t="str"/>
       <x:c r="O31" s="67" t="str"/>
+      <x:c r="P31" s="37"/>
     </x:row>
     <x:row r="32" ht="30" customHeight="1">
       <x:c r="A32" s="20"/>
@@ -1192,11 +1235,12 @@
       <x:c r="M32" s="41"/>
       <x:c r="N32" s="65" t="str"/>
       <x:c r="O32" s="67" t="str"/>
+      <x:c r="P32" s="38"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R211593821c004806"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28d69f555f2b447a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1223,6 +1267,7 @@
     <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="16" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="26" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1259,7 +1304,7 @@
     </x:row>
     <x:row r="3" ht="32" customHeight="1">
       <x:c r="A3" s="44" t="str">
-        <x:v>示例：客户迪奇，仓库 A，尺寸 cm，币种 CNY；入库时间按每行填写，不再另选基准日期。</x:v>
+        <x:v>示例：尺寸 cm，币种 CNY。客户列选填，空白时使用页面默认客户；两处都未填时按未指定客户入账。</x:v>
       </x:c>
       <x:c r="B3" s="44"/>
       <x:c r="C3" s="44"/>
@@ -1291,7 +1336,7 @@
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="6" t="str">
-        <x:v>PO</x:v>
+        <x:v>合同号</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
         <x:v>货号</x:v>
@@ -1334,6 +1379,9 @@
       </x:c>
       <x:c r="O5" s="68" t="str">
         <x:v>入库时间</x:v>
+      </x:c>
+      <x:c r="P5" s="69" t="str">
+        <x:v>客户</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
@@ -1381,6 +1429,9 @@
       </x:c>
       <x:c r="O6" s="67" t="n">
         <x:v>46254.395833333336</x:v>
+      </x:c>
+      <x:c r="P6" s="70" t="str">
+        <x:v>迪奇</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -1421,6 +1472,7 @@
       <x:c r="O7" s="67" t="n">
         <x:v>46255</x:v>
       </x:c>
+      <x:c r="P7" s="70"/>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
       <x:c r="A8" s="22" t="str">
@@ -1465,6 +1517,9 @@
       </x:c>
       <x:c r="O8" s="67" t="n">
         <x:v>46256</x:v>
+      </x:c>
+      <x:c r="P8" s="70" t="str">
+        <x:v>迪奇</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -1503,6 +1558,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="O9" s="67"/>
+      <x:c r="P9" s="70"/>
     </x:row>
     <x:row r="10">
       <x:c r="N10" s="65" t="str"/>
@@ -1510,7 +1566,7 @@
     </x:row>
     <x:row r="11" ht="32" customHeight="1">
       <x:c r="A11" s="1" t="str">
-        <x:v>先选择批次信息，再上传主表。只填基准日实际剩余数量，不填历史入库数或累计出库数。</x:v>
+        <x:v>客户在末列选填，可按行填写不同客户；仓库和尺寸单位按实际资料核实。只填实际剩余结余，不重放历史累计入库。</x:v>
       </x:c>
       <x:c r="B11" s="1"/>
       <x:c r="C11" s="1"/>
@@ -1568,7 +1624,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a3d5915f1044adc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R422445b8939446ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1637,13 +1693,13 @@
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
       <x:c r="A7" s="55" t="str">
-        <x:v>PO、货号</x:v>
+        <x:v>合同号、货号</x:v>
       </x:c>
       <x:c r="B7" s="52" t="str">
         <x:v>按原库存表填写；已设置为文本，保留前导0。</x:v>
       </x:c>
       <x:c r="C7" s="52" t="str">
-        <x:v>用于识别实际库存，不填虚构合同或货号。</x:v>
+        <x:v>用于识别实际库存，不虚构合同或编号；旧模板“PO”列仍可识别。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
@@ -1816,6 +1872,17 @@
       <x:c r="B23" s="2"/>
       <x:c r="C23" s="2"/>
     </x:row>
+    <x:row r="24" ht="52" customHeight="1">
+      <x:c r="A24" s="2" t="str">
+        <x:v>客户（选填）</x:v>
+      </x:c>
+      <x:c r="B24" s="71" t="str">
+        <x:v>在末列“客户”填写本厂已启用的客户名称；留空时使用页面默认客户。</x:v>
+      </x:c>
+      <x:c r="C24" s="71" t="str">
+        <x:v>文件客户和页面默认客户均未填时，按“未指定客户”入账；同表可填写多个客户，不自动新增客户。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>